<commit_message>
fix(fixture): corregir fechas de fase final (R32→Final)
Reescribe el calendario de eliminatorias en el scraper con las fechas
reales (R32 28-jun a 3-jul, etc.) y agrega workflow+script
fix_knockout_dates.mjs para reparar datetime/closesAtMs en Firebase.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mundial_2026_v2.xlsx
+++ b/mundial_2026_v2.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -51,7 +48,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -59,19 +56,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3181,12 +3172,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T13:00</t>
+          <t>2026-06-28T13:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T17:00</t>
+          <t>2026-06-28T17:00</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3209,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T17:00</t>
+          <t>2026-06-29T13:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T21:00</t>
+          <t>2026-06-29T17:00</t>
         </is>
       </c>
     </row>
@@ -3255,12 +3246,12 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T21:00</t>
+          <t>2026-06-29T16:30</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T01:00</t>
+          <t>2026-06-29T20:30</t>
         </is>
       </c>
     </row>
@@ -3292,12 +3283,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T13:00</t>
+          <t>2026-06-29T21:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:00</t>
+          <t>2026-06-30T01:00</t>
         </is>
       </c>
     </row>
@@ -3329,12 +3320,12 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:00</t>
+          <t>2026-06-30T13:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T21:00</t>
+          <t>2026-06-30T17:00</t>
         </is>
       </c>
     </row>
@@ -3366,12 +3357,12 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T21:00</t>
+          <t>2026-06-30T17:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T01:00</t>
+          <t>2026-06-30T21:00</t>
         </is>
       </c>
     </row>
@@ -3403,12 +3394,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T13:00</t>
+          <t>2026-06-30T21:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00</t>
+          <t>2026-07-01T01:00</t>
         </is>
       </c>
     </row>
@@ -3440,12 +3431,12 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00</t>
+          <t>2026-07-01T14:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T21:00</t>
+          <t>2026-07-01T18:00</t>
         </is>
       </c>
     </row>
@@ -3477,12 +3468,12 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T21:00</t>
+          <t>2026-07-01T17:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T01:00</t>
+          <t>2026-07-01T21:00</t>
         </is>
       </c>
     </row>
@@ -3514,12 +3505,12 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T13:00</t>
+          <t>2026-07-01T20:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T17:00</t>
+          <t>2026-07-02T00:00</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3542,12 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T17:00</t>
+          <t>2026-07-02T15:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T21:00</t>
+          <t>2026-07-02T19:00</t>
         </is>
       </c>
     </row>
@@ -3588,12 +3579,12 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04T21:00</t>
+          <t>2026-07-02T16:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T01:00</t>
+          <t>2026-07-02T20:00</t>
         </is>
       </c>
     </row>
@@ -3625,12 +3616,12 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T13:00</t>
+          <t>2026-07-02T19:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T17:00</t>
+          <t>2026-07-02T23:00</t>
         </is>
       </c>
     </row>
@@ -3662,12 +3653,12 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T17:00</t>
+          <t>2026-07-03T13:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T21:00</t>
+          <t>2026-07-03T17:00</t>
         </is>
       </c>
     </row>
@@ -3699,12 +3690,12 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05T21:00</t>
+          <t>2026-07-03T15:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06T01:00</t>
+          <t>2026-07-03T19:00</t>
         </is>
       </c>
     </row>
@@ -3736,12 +3727,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:00</t>
+          <t>2026-07-03T20:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06T21:00</t>
+          <t>2026-07-04T00:00</t>
         </is>
       </c>
     </row>
@@ -3773,12 +3764,12 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T17:00</t>
+          <t>2026-07-04T13:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T21:00</t>
+          <t>2026-07-04T17:00</t>
         </is>
       </c>
     </row>
@@ -3810,12 +3801,12 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T21:00</t>
+          <t>2026-07-04T17:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10T01:00</t>
+          <t>2026-07-04T21:00</t>
         </is>
       </c>
     </row>
@@ -3847,12 +3838,12 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10T17:00</t>
+          <t>2026-07-05T16:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10T21:00</t>
+          <t>2026-07-05T20:00</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3875,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10T21:00</t>
+          <t>2026-07-05T20:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11T01:00</t>
+          <t>2026-07-06T00:00</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3912,12 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11T17:00</t>
+          <t>2026-07-06T15:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11T21:00</t>
+          <t>2026-07-06T19:00</t>
         </is>
       </c>
     </row>
@@ -3958,12 +3949,12 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11T21:00</t>
+          <t>2026-07-06T17:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12T01:00</t>
+          <t>2026-07-06T21:00</t>
         </is>
       </c>
     </row>
@@ -3995,12 +3986,12 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12T17:00</t>
+          <t>2026-07-07T12:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12T21:00</t>
+          <t>2026-07-07T16:00</t>
         </is>
       </c>
     </row>
@@ -4032,12 +4023,12 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12T21:00</t>
+          <t>2026-07-07T16:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13T01:00</t>
+          <t>2026-07-07T20:00</t>
         </is>
       </c>
     </row>
@@ -4069,12 +4060,12 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16T17:00</t>
+          <t>2026-07-09T16:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16T21:00</t>
+          <t>2026-07-09T20:00</t>
         </is>
       </c>
     </row>
@@ -4106,12 +4097,12 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16T21:00</t>
+          <t>2026-07-10T15:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17T01:00</t>
+          <t>2026-07-10T19:00</t>
         </is>
       </c>
     </row>
@@ -4143,12 +4134,12 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17T17:00</t>
+          <t>2026-07-11T17:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17T21:00</t>
+          <t>2026-07-11T21:00</t>
         </is>
       </c>
     </row>
@@ -4180,12 +4171,12 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17T21:00</t>
+          <t>2026-07-11T21:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18T01:00</t>
+          <t>2026-07-12T01:00</t>
         </is>
       </c>
     </row>
@@ -4217,12 +4208,12 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21T21:00</t>
+          <t>2026-07-14T15:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22T01:00</t>
+          <t>2026-07-14T19:00</t>
         </is>
       </c>
     </row>
@@ -4254,12 +4245,12 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22T21:00</t>
+          <t>2026-07-15T15:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23T01:00</t>
+          <t>2026-07-15T19:00</t>
         </is>
       </c>
     </row>
@@ -4286,17 +4277,17 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Sede por confirmar</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T20:00</t>
+          <t>2026-07-18T17:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>2026-07-26T00:00</t>
+          <t>2026-07-18T21:00</t>
         </is>
       </c>
     </row>
@@ -4328,12 +4319,12 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-07-19T20:00</t>
+          <t>2026-07-19T15:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00</t>
+          <t>2026-07-19T19:00</t>
         </is>
       </c>
     </row>

</xml_diff>